<commit_message>
added 5 files and converted
</commit_message>
<xml_diff>
--- a/metadata.xlsx
+++ b/metadata.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="105">
   <si>
     <t>Last Name</t>
   </si>
@@ -285,12 +285,93 @@
   <si>
     <t>473.01 Fall 2018 Transcription Exercise.docx</t>
   </si>
+  <si>
+    <t>O'Driscoll</t>
+  </si>
+  <si>
+    <t>Mike</t>
+  </si>
+  <si>
+    <t>mo@ualberta.ca</t>
+  </si>
+  <si>
+    <t>Alberta, U. of</t>
+  </si>
+  <si>
+    <t>How Poems Work: Introduction to Poetry Winter Term 2023</t>
+  </si>
+  <si>
+    <t>ENGL 206 Syllabus Final(2)-1.md</t>
+  </si>
+  <si>
+    <t>Course: ENGL 483 LEC B1 - Winter 2025 - LITERARY SOUND STUDIES | eClass</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">ENGL 483 eClass </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF000000"/>
+      </rPr>
+      <t>Version.md</t>
+    </r>
+  </si>
+  <si>
+    <t>ENGL 483, Section B1: Literary Sound Studies Department of English and Film Studies Winter Term 2025</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">ENGL 483 </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF000000"/>
+      </rPr>
+      <t>Syllabus-3-1.md</t>
+    </r>
+  </si>
+  <si>
+    <t>Course: ENGL 206 LEC B1 - Winter 2023 - INTRODUCTION TO POETRY | eClass</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">ENGL 206 eClass </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF000000"/>
+      </rPr>
+      <t>Version.md</t>
+    </r>
+  </si>
+  <si>
+    <t>Department of English and Film Studies ENGL 569 A1: Ethical Listening Fall Term 2022</t>
+  </si>
+  <si>
+    <t>Syllabus ENGL 569 Ethical Listening(1)(1)(1).md</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -311,6 +392,11 @@
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -326,7 +412,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -344,6 +430,12 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1683,6 +1775,30 @@
       <c r="AD23" s="3"/>
     </row>
     <row r="24">
+      <c r="A24" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
       <c r="M24" s="3"/>
@@ -1705,6 +1821,30 @@
       <c r="AD24" s="3"/>
     </row>
     <row r="25">
+      <c r="A25" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
@@ -1727,6 +1867,30 @@
       <c r="AD25" s="3"/>
     </row>
     <row r="26">
+      <c r="A26" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
@@ -1749,6 +1913,30 @@
       <c r="AD26" s="3"/>
     </row>
     <row r="27">
+      <c r="A27" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
@@ -1771,6 +1959,30 @@
       <c r="AD27" s="3"/>
     </row>
     <row r="28">
+      <c r="A28" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>

</xml_diff>